<commit_message>
Upgraded miniature setup screens and management features.
</commit_message>
<xml_diff>
--- a/.deploy/frontend-iis/templates/Bulk Upload Miniature Template.xlsx
+++ b/.deploy/frontend-iis/templates/Bulk Upload Miniature Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Development\Source\RPG Collection Navigator\frontend\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0DC05CF4-FA06-436A-B8C8-D03C6286005A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAF1528A-F025-44F4-A27A-4A7589889986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3600" yWindow="2685" windowWidth="31170" windowHeight="15990" xr2:uid="{2FC99663-8B02-44A8-96B9-B2E56A19E978}"/>
+    <workbookView xWindow="19875" yWindow="2415" windowWidth="31170" windowHeight="15990" xr2:uid="{2FC99663-8B02-44A8-96B9-B2E56A19E978}"/>
   </bookViews>
   <sheets>
     <sheet name="Bulk Upload File" sheetId="1" r:id="rId1"/>
@@ -22,12 +22,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
-    <t>Collection</t>
-  </si>
-  <si>
-    <t>Sub Category</t>
-  </si>
-  <si>
     <t>Miniature Name</t>
   </si>
   <si>
@@ -38,6 +32,12 @@
   </si>
   <si>
     <t>Item</t>
+  </si>
+  <si>
+    <t>Size</t>
+  </si>
+  <si>
+    <t>Rarity</t>
   </si>
 </sst>
 </file>
@@ -902,11 +902,9 @@
   <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.42578125" customWidth="1"/>
+    <col min="1" max="1" width="19.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="18.42578125" customWidth="1"/>
     <col min="6" max="6" width="8.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -915,22 +913,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>2</v>
-      </c>
-      <c r="E1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" t="s">
-        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>